<commit_message>
Add follow-up for Johannes (B08T9TBC4C)
</commit_message>
<xml_diff>
--- a/2026-04-15_B08T9TBC4C/B08T9TBC4C_magnesium_kapseln_bulksheet.xlsx
+++ b/2026-04-15_B08T9TBC4C/B08T9TBC4C_magnesium_kapseln_bulksheet.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>BODYLAB-CMG-120</t>
+          <t>B08T9TBC4C</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>BODYLAB-CMG-120</t>
+          <t>B08T9TBC4C</t>
         </is>
       </c>
     </row>

</xml_diff>